<commit_message>
cli module added project structure refactored adapter layer added
</commit_message>
<xml_diff>
--- a/src/jira_crawler/output/test.xlsx
+++ b/src/jira_crawler/output/test.xlsx
@@ -10,50 +10,56 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
   <si>
     <t>Export Format: CSV / XLSX
 Template Version: 1.0
-Generated On: 2026-05-31 21:25:23</t>
-  </si>
-  <si>
-    <t>CAMEL-23239</t>
-  </si>
-  <si>
-    <t>Addcamel-state-storecomponentwithpluggablekey-valuestore</t>
-  </si>
-  <si>
-    <t>NewFeature</t>
-  </si>
-  <si>
-    <t>InProgress</t>
-  </si>
-  <si>
-    <t>Major</t>
-  </si>
-  <si>
-    <t>Unresolved</t>
-  </si>
-  <si>
-    <t>GuillaumeNodet</t>
-  </si>
-  <si>
-    <t>2026-03-24T10:30:49+0000</t>
-  </si>
-  <si>
-    <t>1774348249</t>
-  </si>
-  <si>
-    <t>2026-05-29T20:40:00+0000</t>
-  </si>
-  <si>
-    <t>1780087200</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>&lt;divclass="user-content-block"&gt;&lt;h2&gt;&lt;aname="Motivation"&gt;&lt;/a&gt;Motivation&lt;/h2&gt;&lt;p&gt;Camelprovidesdedicatedcomponentsforspecificcaching/storetechnologies(Caffeine,Redis,Infinispan,etc.),eachwithitsownAPIsurface.Thisworkswellwhenusersneedthefullfeaturesetofaspecifictechnology,butitcreatesfrictionwhentheactualneedissimple:storeandretrievekey-valuepairs.&lt;/p&gt;&lt;p&gt;The&lt;tt&gt;camel-state-store&lt;/tt&gt;componentfollowsthesame&amp;#34;choosetheproblem,notthetechnology&amp;#34;patternthatCamelalreadyusessuccessfullyinotherareas:&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;tt&gt;camel-sql&lt;/tt&gt;/&lt;tt&gt;camel-jdbc&lt;/tt&gt;—genericSQLoveranyJDBCdatabase,withoutlockingintoavendor&lt;/li&gt;&lt;li&gt;&lt;tt&gt;camel-jms&lt;/tt&gt;—genericmessagingoveranyJMSprovider(with&lt;tt&gt;camel-activemq&lt;/tt&gt;,&lt;tt&gt;camel-amqp&lt;/tt&gt;aspre-configuredvariants)&lt;/li&gt;&lt;li&gt;&lt;tt&gt;camel-jcache&lt;/tt&gt;—genericcachingviaJSR-107overanycompliantimplementation&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;Similarly,&lt;tt&gt;camel-state-store&lt;/tt&gt;providesaunifiedkey-valueAPIwhere:&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Userschoosethecapabilityfirst(&amp;#34;Ineedakey-valuestore&amp;#34;)ratherthanaspecifictechnology&lt;/li&gt;&lt;li&gt;Thebackendisswappablewithoutchangingroutelogic—developwithin-memory,deploywithRedisorInfinispan&lt;/li&gt;&lt;li&gt;TheAPIsurfaceisintentionallyminimal(put,get,delete,contains,keys,clear)—unlikethefull-featuredtechnology-specificcomponents&lt;/li&gt;&lt;/ul&gt;&lt;h2&gt;&lt;aname="Differencefromexistingcachecomponents"&gt;&lt;/a&gt;Differencefromexistingcachecomponents&lt;/h2&gt;&lt;divclass="table-wrap"&gt;&lt;tableclass="confluenceTable"&gt;&lt;tbody&gt;&lt;tr&gt;&lt;thclass="confluenceTh"&gt;&lt;/th&gt;&lt;thclass="confluenceTh"&gt;camel-state-store&lt;/th&gt;&lt;thclass="confluenceTh"&gt;camel-caffeine-cache/camel-infinispan/etc.&lt;/th&gt;&lt;/tr&gt;&lt;tr&gt;&lt;tdclass="confluenceTd"&gt;&lt;b&gt;Focus&lt;/b&gt;&lt;/td&gt;&lt;tdclass="confluenceTd"&gt;Simplekey-valuestoreabstraction&lt;/td&gt;&lt;tdclass="confluenceTd"&gt;Fullfeaturesetofaspecifictechnology&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;tdclass="confluenceTd"&gt;&lt;b&gt;Backend&lt;/b&gt;&lt;/td&gt;&lt;tdclass="confluenceTd"&gt;Pluggablevia&lt;tt&gt;StateStoreBackend&lt;/tt&gt;interface&lt;/td&gt;&lt;tdclass="confluenceTd"&gt;Fixedtoonetechnology&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;tdclass="confluenceTd"&gt;&lt;b&gt;API&lt;/b&gt;&lt;/td&gt;&lt;tdclass="confluenceTd"&gt;Minimal:put,get,delete,contains,keys,clear&lt;/td&gt;&lt;tdclass="confluenceTd"&gt;Rich:queries,events,statistics,pub/sub,etc.&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;tdclass="confluenceTd"&gt;&lt;b&gt;Usecase&lt;/b&gt;&lt;/td&gt;&lt;tdclass="confluenceTd"&gt;Portability,simplicity,migrationfromMuleSoftObjectStore&lt;/td&gt;&lt;tdclass="confluenceTd"&gt;Deepintegrationwithaspecificproduct&lt;/td&gt;&lt;/tr&gt;&lt;/tbody&gt;&lt;/table&gt;&lt;/div&gt;&lt;h2&gt;&lt;aname="Features"&gt;&lt;/a&gt;Features&lt;/h2&gt;&lt;ul&gt;&lt;li&gt;New&lt;tt&gt;camel-state-store&lt;/tt&gt;componentprovidingasimple,unifiedkey-valuestoreAPIwithpluggablebackends&lt;/li&gt;&lt;li&gt;Supportsoperations:&lt;tt&gt;put&lt;/tt&gt;,&lt;tt&gt;putIfAbsent&lt;/tt&gt;,&lt;tt&gt;get&lt;/tt&gt;,&lt;tt&gt;delete&lt;/tt&gt;,&lt;tt&gt;contains&lt;/tt&gt;,&lt;tt&gt;keys&lt;/tt&gt;,&lt;tt&gt;size&lt;/tt&gt;,&lt;tt&gt;clear&lt;/tt&gt;&lt;/li&gt;&lt;li&gt;Per-entryTTLwithendpoint-leveldefaultandper-messageoverridevia&lt;tt&gt;CamelStateStoreTtl&lt;/tt&gt;header&lt;/li&gt;&lt;li&gt;&lt;b&gt;Auto-discovery&lt;/b&gt;:ifasingle&lt;tt&gt;StateStoreBackend&lt;/tt&gt;beanisintheregistry,itisusedautomatically—no&lt;tt&gt;backend=#beanName&lt;/tt&gt;neededonendpoints.LogsaWARNwhenmultiplebackendsarefound.&lt;/li&gt;&lt;li&gt;&lt;b&gt;Property-basedconfiguration&lt;/b&gt;:backendscanbefullyconfiguredvia&lt;tt&gt;application.properties&lt;/tt&gt;using&lt;tt&gt;camel.beans.*&lt;/tt&gt;syntax—noJavacoderequired&lt;/li&gt;&lt;li&gt;Multi-modulestructurewithpluggablebackends:&lt;ul&gt;&lt;li&gt;&lt;tt&gt;camel-state-store&lt;/tt&gt;:core+in-memorybackend(&lt;tt&gt;ConcurrentHashMap&lt;/tt&gt;,lazyTTL)&lt;/li&gt;&lt;li&gt;&lt;tt&gt;camel-state-store-caffeine&lt;/tt&gt;:Caffeinecachewithper-entryvariableexpiry&lt;/li&gt;&lt;li&gt;&lt;tt&gt;camel-state-store-redis&lt;/tt&gt;:Redisson&lt;tt&gt;RMapCache&lt;/tt&gt;withnativeTTL&lt;/li&gt;&lt;li&gt;&lt;tt&gt;camel-state-store-infinispan&lt;/tt&gt;:HotRodclientwithlifespanTTL&lt;/li&gt;&lt;/ul&gt;&lt;/li&gt;&lt;li&gt;Custombackendsvia&lt;tt&gt;StateStoreBackend&lt;/tt&gt;interfaceandbeanreferences&lt;/li&gt;&lt;li&gt;Thread-safebackendlifecycle:&lt;tt&gt;start()&lt;/tt&gt;calledonceperbackend,idempotentguardsinallbackends&lt;/li&gt;&lt;/ul&gt;&lt;h2&gt;&lt;aname="Routeexamples"&gt;&lt;/a&gt;Routeexamples&lt;/h2&gt;&lt;h3&gt;&lt;aname="Simpleput%2Fgetwithinmemorybackend"&gt;&lt;/a&gt;Simpleput/getwithin-memorybackend&lt;/h3&gt;&lt;divclass="codepanel"style="border-width:1px;"&gt;&lt;divclass="codeContentpanelContent"&gt;&lt;preclass="code-java"&gt;from(&lt;spanclass="code-quote"&gt;&amp;#34;direct:store&amp;#34;&lt;/span&gt;).setHeader(StateStoreConstants.KEY,constant(&lt;spanclass="code-quote"&gt;&amp;#34;user-123&amp;#34;&lt;/span&gt;)).to(&lt;spanclass="code-quote"&gt;&amp;#34;state-store:sessions?operation=put&amp;#34;&lt;/span&gt;);from(&lt;spanclass="code-quote"&gt;&amp;#34;direct:lookup&amp;#34;&lt;/span&gt;).setHeader(StateStoreConstants.KEY,constant(&lt;spanclass="code-quote"&gt;&amp;#34;user-123&amp;#34;&lt;/span&gt;)).to(&lt;spanclass="code-quote"&gt;&amp;#34;state-store:sessions?operation=get&amp;#34;&lt;/span&gt;).log(&lt;spanclass="code-quote"&gt;&amp;#34;Found:${body}&amp;#34;&lt;/span&gt;);&lt;/pre&gt;&lt;/div&gt;&lt;/div&gt;&lt;h3&gt;&lt;aname="CachingHTTPresponseswithTTL"&gt;&lt;/a&gt;CachingHTTPresponseswithTTL&lt;/h3&gt;&lt;divclass="codepanel"style="border-width:1px;"&gt;&lt;divclass="codeContentpanelContent"&gt;&lt;preclass="code-java"&gt;from(&lt;spanclass="code-quote"&gt;&amp;#34;timer:poll?period=60000&amp;#34;&lt;/span&gt;).setHeader(StateStoreConstants.KEY,constant(&lt;spanclass="code-quote"&gt;&amp;#34;weather&amp;#34;&lt;/span&gt;)).to(&lt;spanclass="code-quote"&gt;&amp;#34;state-store:cache?operation=get&amp;#34;&lt;/span&gt;).choice().when(body().isNull()).to(&lt;spanclass="code-quote"&gt;&amp;#34;https:&lt;spanclass="code-comment"&gt;//api.weather.com/current&amp;#34;&lt;/span&gt;)&lt;/span&gt;.setHeader(StateStoreConstants.KEY,constant(&lt;spanclass="code-quote"&gt;&amp;#34;weather&amp;#34;&lt;/span&gt;)).setHeader(StateStoreConstants.TTL,constant(300000L)).to(&lt;spanclass="code-quote"&gt;&amp;#34;state-store:cache?operation=put&amp;#34;&lt;/span&gt;).end().to(&lt;spanclass="code-quote"&gt;&amp;#34;direct:process-weather&amp;#34;&lt;/span&gt;);&lt;/pre&gt;&lt;/div&gt;&lt;/div&gt;&lt;h3&gt;&lt;aname="Idempotentdeduplicationpattern"&gt;&lt;/a&gt;Idempotentdeduplicationpattern&lt;/h3&gt;&lt;divclass="codepanel"style="border-width:1px;"&gt;&lt;divclass="codeContentpanelContent"&gt;&lt;preclass="code-java"&gt;from(&lt;spanclass="code-quote"&gt;&amp;#34;kafka:orders&amp;#34;&lt;/span&gt;).setHeader(StateStoreConstants.KEY,simple(&lt;spanclass="code-quote"&gt;&amp;#34;${header.orderId}&amp;#34;&lt;/span&gt;)).to(&lt;spanclass="code-quote"&gt;&amp;#34;state-store:processed?operation=putIfAbsent&amp;#34;&lt;/span&gt;).choice().when(body().isNotNull()).log(&lt;spanclass="code-quote"&gt;&amp;#34;Duplicateorder${header.orderId},skipping&amp;#34;&lt;/span&gt;).stop().end().to(&lt;spanclass="code-quote"&gt;&amp;#34;direct:process-order&amp;#34;&lt;/span&gt;);&lt;/pre&gt;&lt;/div&gt;&lt;/div&gt;&lt;h3&gt;&lt;aname="YAMLDSLwithpropertyconfiguredRedisbackend"&gt;&lt;/a&gt;YAMLDSLwithproperty-configuredRedisbackend&lt;/h3&gt;&lt;divclass="codepanel"style="border-width:1px;"&gt;&lt;divclass="codeHeaderpanelHeader"style="border-bottom-width:1px;"&gt;&lt;b&gt;application.properties&lt;/b&gt;&lt;/div&gt;&lt;divclass="codeContentpanelContent"&gt;&lt;preclass="code-java"&gt;camel.beans.redisBackend=#&lt;spanclass="code-keyword"&gt;class:&lt;/span&gt;org.apache.camel.component.statestore.redis.RedisStateStoreBackendcamel.beans.redisBackend.redisUrl=redis:&lt;spanclass="code-comment"&gt;//redis:6379&lt;/span&gt;camel.beans.redisBackend.mapName=app-state&lt;/pre&gt;&lt;/div&gt;&lt;/div&gt;&lt;divclass="codepanel"style="border-width:1px;"&gt;&lt;divclass="codeContentpanelContent"&gt;&lt;preclass="code-yaml"&gt;-&lt;spanclass="code-keyword"&gt;route:&lt;/span&gt;&lt;spanclass="code-keyword"&gt;from:&lt;/span&gt;&lt;spanclass="code-keyword"&gt;uri:&lt;/span&gt;direct:save&lt;spanclass="code-keyword"&gt;steps:&lt;/span&gt;-&lt;spanclass="code-keyword"&gt;setHeader:&lt;/span&gt;&lt;spanclass="code-keyword"&gt;name:&lt;/span&gt;CamelStateStoreKey&lt;spanclass="code-keyword"&gt;simple:&lt;/span&gt;&lt;spanclass="code-quote"&gt;&amp;#34;${header.userId}&amp;#34;&lt;/span&gt;-&lt;spanclass="code-keyword"&gt;to:&lt;/span&gt;&lt;spanclass="code-keyword"&gt;uri:&lt;/span&gt;state-store:preferences?operation=put-&lt;spanclass="code-keyword"&gt;route:&lt;/span&gt;&lt;spanclass="code-keyword"&gt;from:&lt;/span&gt;&lt;spanclass="code-keyword"&gt;uri:&lt;/span&gt;direct:load&lt;spanclass="code-keyword"&gt;steps:&lt;/span&gt;-&lt;spanclass="code-keyword"&gt;setHeader:&lt;/span&gt;&lt;spanclass="code-keyword"&gt;name:&lt;/span&gt;CamelStateStoreKey&lt;spanclass="code-keyword"&gt;simple:&lt;/span&gt;&lt;spanclass="code-quote"&gt;&amp;#34;${header.userId}&amp;#34;&lt;/span&gt;-&lt;spanclass="code-keyword"&gt;to:&lt;/span&gt;&lt;spanclass="code-keyword"&gt;uri:&lt;/span&gt;state-store:preferences?operation=get&lt;/pre&gt;&lt;/div&gt;&lt;/div&gt;&lt;h2&gt;&lt;aname="Configurationexamples"&gt;&lt;/a&gt;Configurationexamples&lt;/h2&gt;&lt;h3&gt;&lt;aname="Javabeanregistration"&gt;&lt;/a&gt;Javabeanregistration&lt;/h3&gt;&lt;divclass="codepanel"style="border-width:1px;"&gt;&lt;divclass="codeContentpanelContent"&gt;&lt;preclass="code-java"&gt;@BindToRegistry(&lt;spanclass="code-quote"&gt;&amp;#34;caffeineBackend&amp;#34;&lt;/span&gt;)&lt;spanclass="code-keyword"&gt;public&lt;/span&gt;CaffeineStateStoreBackendcaffeine(){CaffeineStateStoreBackendbackend=&lt;spanclass="code-keyword"&gt;new&lt;/span&gt;CaffeineStateStoreBackend();backend.setMaximumSize(50_000);&lt;spanclass="code-keyword"&gt;return&lt;/span&gt;backend;}&lt;/pre&gt;&lt;/div&gt;&lt;/div&gt;&lt;h3&gt;&lt;aname="Propertybasedconfiguration%28noJavarequired%29"&gt;&lt;/a&gt;Property-basedconfiguration(noJavarequired)&lt;/h3&gt;&lt;divclass="codepanel"style="border-width:1px;"&gt;&lt;divclass="codeHeaderpanelHeader"style="border-bottom-width:1px;"&gt;&lt;b&gt;Caffeine&lt;/b&gt;&lt;/div&gt;&lt;divclass="codeContentpanelContent"&gt;&lt;preclass="code-java"&gt;camel.beans.caffeineBackend=#&lt;spanclass="code-keyword"&gt;class:&lt;/span&gt;org.apache.camel.component.statestore.caffeine.CaffeineStateStoreBackendcamel.beans.caffeineBackend.maximumSize=50000&lt;/pre&gt;&lt;/div&gt;&lt;/div&gt;&lt;divclass="codepanel"style="border-width:1px;"&gt;&lt;divclass="codeHeaderpanelHeader"style="border-bottom-width:1px;"&gt;&lt;b&gt;Redis&lt;/b&gt;&lt;/div&gt;&lt;divclass="codeContentpanelContent"&gt;&lt;preclass="code-java"&gt;camel.beans.redisBackend=#&lt;spanclass="code-keyword"&gt;class:&lt;/span&gt;org.apache.camel.component.statestore.redis.RedisStateStoreBackendcamel.beans.redisBackend.redisUrl=redis:&lt;spanclass="code-comment"&gt;//myhost:6379&lt;/span&gt;camel.beans.redisBackend.mapName=my-app-state&lt;/pre&gt;&lt;/div&gt;&lt;/div&gt;&lt;divclass="codepanel"style="border-width:1px;"&gt;&lt;divclass="codeHeaderpanelHeader"style="border-bottom-width:1px;"&gt;&lt;b&gt;Infinispan&lt;/b&gt;&lt;/div&gt;&lt;divclass="codeContentpanelContent"&gt;&lt;preclass="code-java"&gt;camel.beans.infinispanBackend=#&lt;spanclass="code-keyword"&gt;class:&lt;/span&gt;org.apache.camel.component.statestore.infinispan.InfinispanStateStoreBackendcamel.beans.infinispanBackend.hosts=myhost:11222camel.beans.infinispanBackend.cacheName=my-cache&lt;/pre&gt;&lt;/div&gt;&lt;/div&gt;&lt;h2&gt;&lt;aname="Designdecision%3AStateStoreBackendinterfacelocation"&gt;&lt;/a&gt;Designdecision:StateStoreBackendinterfacelocation&lt;/h2&gt;&lt;p&gt;Weconsideredmovingthe&lt;tt&gt;StateStoreBackend&lt;/tt&gt;interfaceto&lt;tt&gt;camel-api&lt;/tt&gt;alongsideexistingSPIs(&lt;tt&gt;IdempotentRepository&lt;/tt&gt;,&lt;tt&gt;AggregationRepository&lt;/tt&gt;,&lt;tt&gt;StateRepository&lt;/tt&gt;).Wedecidedagainstitbecause:&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Theexisting&lt;tt&gt;camel-api&lt;/tt&gt;SPIsaretherebecausecoreEIPsconsumethem(idempotentconsumer,aggregator).&lt;tt&gt;StateStoreBackend&lt;/tt&gt;isonlyconsumedbythecomponentitself.&lt;/li&gt;&lt;li&gt;TheexistingSPIshavedifferentsemantics(two-phaseconfirm/rollback,Exchangeserialization)thatdon&amp;#39;tmaptoasimplekey-valuestore.&lt;/li&gt;&lt;li&gt;MovingitwouldaddAPIsurfacewithstricterstabilityguaranteesfornopracticalbenefittoday.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;IfafuturecoreEIPneedsagenerickey-valuestore,theinterfacecanbepromotedthen.&lt;/p&gt;&lt;/div&gt;</t>
+Generated On: 2026-05-31 22:57:06</t>
+  </si>
+  <si>
+    <t>CAMEL-10597</t>
+  </si>
+  <si>
+    <t>Swaggerprintschildobjecttypesasstringparametersratherthanrefs</t>
+  </si>
+  <si>
+    <t>Bug</t>
+  </si>
+  <si>
+    <t>Resolved</t>
+  </si>
+  <si>
+    <t>Minor</t>
+  </si>
+  <si>
+    <t>Fixed</t>
+  </si>
+  <si>
+    <t>ClausIbsen</t>
+  </si>
+  <si>
+    <t>BobPaulin</t>
+  </si>
+  <si>
+    <t>2016-12-14T14:42:08+0000</t>
+  </si>
+  <si>
+    <t>1481726528</t>
+  </si>
+  <si>
+    <t>2016-12-15T14:26:13+0000</t>
+  </si>
+  <si>
+    <t>1481811973</t>
+  </si>
+  <si>
+    <t>2016-12-14T15:31:58+0000</t>
+  </si>
+  <si>
+    <t>1481729518</t>
+  </si>
+  <si>
+    <t>&lt;divclass="user-content-block"&gt;&lt;p&gt;AssumeIhaverestpath&lt;/p&gt;&lt;divclass="codepanel"style="border-width:1px;"&gt;&lt;divclass="codeContentpanelContent"&gt;&lt;preclass="code-java"&gt;&lt;spanclass="code-keyword"&gt;rest&lt;/span&gt;(&lt;spanclass="code-quote"&gt;&amp;#34;/test&amp;#34;&lt;/span&gt;).get().type(ClassA.class).to(&lt;spanclass="code-quote"&gt;&amp;#34;direct:someRoute&amp;#34;&lt;/span&gt;);&lt;spanclass="code-keyword"&gt;rest&lt;/span&gt;(&lt;spanclass="code-quote"&gt;&amp;#34;/testSub&amp;#34;&lt;/span&gt;).get().type(ClassB.class).to(&lt;spanclass="code-quote"&gt;&amp;#34;direct:someOtherRoute&amp;#34;&lt;/span&gt;);&lt;/pre&gt;&lt;/div&gt;&lt;/div&gt;&lt;p&gt;AndinthetypeClassAcontainsareferencetoClassB.&lt;/p&gt;&lt;p&gt;WithintheSwaggerDocthepathforClassArendersasexpected:&lt;/p&gt;&lt;divclass="codepanel"style="border-width:1px;"&gt;&lt;divclass="codeContentpanelContent"&gt;&lt;preclass="code-java"&gt;/test:get:responses:200:schema:$ref:&lt;spanclass="code-quote"&gt;&amp;#39;#/definitions/ClassA&amp;#39;&lt;/span&gt;&lt;/pre&gt;&lt;/div&gt;&lt;/div&gt;&lt;p&gt;HoweverClassBgetsastringparameterscheme&lt;/p&gt;&lt;divclass="codepanel"style="border-width:1px;"&gt;&lt;divclass="codeContentpanelContent"&gt;&lt;preclass="code-java"&gt;/testSub:get:responses:200:schema:type:&lt;spanclass="code-quote"&gt;&amp;#39;string&amp;#39;&lt;/span&gt;format:&lt;spanclass="code-quote"&gt;&amp;#39;com.ClassB&amp;#39;&lt;/span&gt;&lt;/pre&gt;&lt;/div&gt;&lt;/div&gt;&lt;p&gt;HoweverI&amp;#39;dexpectittobe:&lt;/p&gt;&lt;divclass="codepanel"style="border-width:1px;"&gt;&lt;divclass="codeContentpanelContent"&gt;&lt;preclass="code-java"&gt;/testSub:get:responses:200:schema:$ref:&lt;spanclass="code-quote"&gt;&amp;#39;#/definitions/ClassB&amp;#39;&lt;/span&gt;&lt;/pre&gt;&lt;/div&gt;&lt;/div&gt;&lt;/div&gt;</t>
   </si>
   <si>
     <t>{{CommentAuthor1}}</t>
@@ -116,19 +122,52 @@
     <t>{{CommentBody5}}</t>
   </si>
   <si>
-    <t>2026-05-23T18:01:52+0000</t>
-  </si>
-  <si>
-    <t>1779559312</t>
-  </si>
-  <si>
-    <t>Wouldbeniceifthekey-valuestoresupportsecrets(likepasswords)thatareencrypted.hasawaytogetthestate-storeasamapobjectprogrammaticallyNote:AtthemomentweuseMongoDB:https://academy.fluxygen.com/docs/4.17.10/components/endpoints/get_tenant_variablehttps://academy.fluxygen.com/docs/4.17.10/components/endpoints/set_tenant_variableMaygivessomeinspiration.WouldbeniceifwecouldreplaceitwithCamelstate-store.WealsouseMapDB,whichisnicetostorevariousobjectoff-heap:https://mapdb.org/Lookingforwardtotrythis.</t>
-  </si>
-  <si>
-    <t>Raymond</t>
-  </si>
-  <si>
-    <t>Also,thiswouldbeanexcellentcandidatetouseincombinationwithvariables:https://camel.apache.org/manual/variables.html</t>
+    <t>GitHubuserbobpaulinopenedapullrequest:https://github.com/apache/camel/pull/1348CAMEL-10597-Allowadditionofx-classNametoemptyVendorExtensionsYoucanmergethispullrequestintoaGitrepositorybyrunning:$gitpullhttps://github.com/bobpaulin/camelCAMEL-10597Alternativelyyoucanreviewandapplythesechangesasthepatchat:https://github.com/apache/camel/pull/1348.patchToclosethispullrequest,makeacommittoyourmaster/trunkbranchwith(atleast)thefollowinginthecommitmessage:Thiscloses#1348</t>
+  </si>
+  <si>
+    <t>ASFGitHubBot</t>
+  </si>
+  <si>
+    <t>2016-12-14T14:55:56+0000</t>
+  </si>
+  <si>
+    <t>1481727356</t>
+  </si>
+  <si>
+    <t>2016-12-14T14:56:06+0000</t>
+  </si>
+  <si>
+    <t>1481727366</t>
+  </si>
+  <si>
+    <t>PRincludedhttps://github.com/apache/camel/pull/1348</t>
+  </si>
+  <si>
+    <t>ThanksforthePR</t>
+  </si>
+  <si>
+    <t>2016-12-14T15:34:04+0000</t>
+  </si>
+  <si>
+    <t>1481729644</t>
+  </si>
+  <si>
+    <t>Githubuserbobpaulinclosedthepullrequestat:https://github.com/apache/camel/pull/1348</t>
+  </si>
+  <si>
+    <t>AndreaCosentino</t>
+  </si>
+  <si>
+    <t>2016-12-15T14:05:25+0000</t>
+  </si>
+  <si>
+    <t>1481810725</t>
+  </si>
+  <si>
+    <t>2.17.xisaffectedtoodavsclaus</t>
+  </si>
+  <si>
+    <t>Thanksitsbackportednow</t>
   </si>
 </sst>
 </file>
@@ -814,7 +853,7 @@
         <v>Reporter</v>
       </c>
       <c r="C14" s="29" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D14" s="29" t="str">
         <v>—</v>
@@ -834,10 +873,10 @@
         <v>Created</v>
       </c>
       <c r="C15" s="32" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D15" s="32" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E15" s="32" t="str">
         <v>Issue creation date</v>
@@ -854,10 +893,10 @@
         <v>Updated</v>
       </c>
       <c r="C16" s="29" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D16" s="29" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E16" s="29" t="str">
         <v>Last update date</v>
@@ -874,10 +913,10 @@
         <v>Resolved</v>
       </c>
       <c r="C17" s="32" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D17" s="32" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E17" s="32" t="str">
         <v>Resolution date</v>
@@ -894,7 +933,7 @@
         <v>Description</v>
       </c>
       <c r="C18" s="54" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D18" s="54" t="str">
         <v>—</v>
@@ -956,10 +995,10 @@
         <v>37</v>
       </c>
       <c r="C22" s="29" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D22" s="29" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="E22" s="29" t="s">
         <v>36</v>
@@ -975,16 +1014,16 @@
         <v>2</v>
       </c>
       <c r="B23" s="29" t="s">
-        <v>37</v>
+        <v>8</v>
       </c>
       <c r="C23" s="29" t="s">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="D23" s="29" t="s">
-        <v>11</v>
+        <v>41</v>
       </c>
       <c r="E23" s="29" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="F23" s="4">
         <v>2</v>
@@ -997,19 +1036,19 @@
         <v>3</v>
       </c>
       <c r="B24" s="29" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C24" s="29" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D24" s="29" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E24" s="29" t="s">
-        <v>12</v>
-      </c>
-      <c r="F24" s="4" t="s">
-        <v>12</v>
+        <v>43</v>
+      </c>
+      <c r="F24" s="4">
+        <v>3</v>
       </c>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -1019,19 +1058,19 @@
         <v>4</v>
       </c>
       <c r="B25" s="29" t="s">
-        <v>12</v>
+        <v>37</v>
       </c>
       <c r="C25" s="29" t="s">
-        <v>12</v>
+        <v>44</v>
       </c>
       <c r="D25" s="29" t="s">
-        <v>12</v>
+        <v>45</v>
       </c>
       <c r="E25" s="29" t="s">
-        <v>12</v>
-      </c>
-      <c r="F25" s="4" t="s">
-        <v>12</v>
+        <v>46</v>
+      </c>
+      <c r="F25" s="4">
+        <v>4</v>
       </c>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -1041,37 +1080,42 @@
         <v>5</v>
       </c>
       <c r="B26" s="29" t="s">
-        <v>12</v>
+        <v>47</v>
       </c>
       <c r="C26" s="29" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="D26" s="29" t="s">
-        <v>12</v>
+        <v>49</v>
       </c>
       <c r="E26" s="29" t="s">
-        <v>12</v>
-      </c>
-      <c r="F26" s="4" t="s">
-        <v>12</v>
+        <v>50</v>
+      </c>
+      <c r="F26" s="4">
+        <v>5</v>
       </c>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
     </row>
-    <row r="27" ht="24" customHeight="true">
-      <c r="A27" s="4"/>
-      <c r="B27" s="4"/>
-      <c r="C27" s="4"/>
-      <c r="D27" s="4"/>
-      <c r="E27" s="4"/>
-      <c r="F27" s="4"/>
-      <c r="G27" s="4"/>
-      <c r="H27" s="4"/>
-    </row>
-    <row r="28" ht="26" customHeight="true">
-      <c r="A28" s="59" t="str">
-        <v>ℹ Note: Epoch timestamps are in milliseconds UTC. Date/time values are displayed in the system default timezone.</v>
-      </c>
+    <row r="27" ht="44" customHeight="true">
+      <c r="B27" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="C27" s="29" t="s">
+        <v>11</v>
+      </c>
+      <c r="D27" s="29" t="s">
+        <v>12</v>
+      </c>
+      <c r="E27" s="29" t="s">
+        <v>51</v>
+      </c>
+      <c r="F27" s="4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="28" ht="24" customHeight="true">
+      <c r="A28" s="4"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -1080,6 +1124,18 @@
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
     </row>
+    <row r="29" ht="26" customHeight="true">
+      <c r="A29" s="59" t="str">
+        <v>ℹ Note: Epoch timestamps are in milliseconds UTC. Date/time values are displayed in the system default timezone.</v>
+      </c>
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="4"/>
+      <c r="H29" s="4"/>
+    </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A1:E1"/>
@@ -1087,16 +1143,16 @@
     <mergeCell ref="F1:H3"/>
     <mergeCell ref="A5:H5"/>
     <mergeCell ref="A20:H20"/>
-    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A29:H29"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation allowBlank="false" sqref="C9" type="list">
+    <dataValidation allowBlank="false" sqref="C9:C9" type="list">
       <formula1>Lists!$C$2:$C$7</formula1>
     </dataValidation>
-    <dataValidation allowBlank="false" sqref="C10" type="list">
+    <dataValidation allowBlank="false" sqref="C10:C10" type="list">
       <formula1>Lists!$A$2:$A$5</formula1>
     </dataValidation>
-    <dataValidation allowBlank="false" sqref="C11" type="list">
+    <dataValidation allowBlank="false" sqref="C11:C11" type="list">
       <formula1>Lists!$B$2:$B$6</formula1>
     </dataValidation>
   </dataValidations>
@@ -1105,432 +1161,432 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="8.75" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="6.059999942779541" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="10.770000457763672" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="63" t="str">
-        <x:v>Status</x:v>
-      </x:c>
-      <x:c r="B1" s="63" t="str">
-        <x:v>Priority</x:v>
-      </x:c>
-      <x:c r="C1" s="63" t="str">
-        <x:v>Type</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" t="str">
-        <x:v>Open</x:v>
-      </x:c>
-      <x:c r="B2" t="str">
-        <x:v>Blocker</x:v>
-      </x:c>
-      <x:c r="C2" t="str">
-        <x:v>Bug</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" t="str">
-        <x:v>In Progress</x:v>
-      </x:c>
-      <x:c r="B3" t="str">
-        <x:v>Critical</x:v>
-      </x:c>
-      <x:c r="C3" t="str">
-        <x:v>Task</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" t="str">
-        <x:v>Resolved</x:v>
-      </x:c>
-      <x:c r="B4" t="str">
-        <x:v>Major</x:v>
-      </x:c>
-      <x:c r="C4" t="str">
-        <x:v>Improvement</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" t="str">
-        <x:v>Closed</x:v>
-      </x:c>
-      <x:c r="B5" t="str">
-        <x:v>Minor</x:v>
-      </x:c>
-      <x:c r="C5" t="str">
-        <x:v>New Feature</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="B6" t="str">
-        <x:v>Trivial</x:v>
-      </x:c>
-      <x:c r="C6" t="str">
-        <x:v>Test</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="C7" t="str">
-        <x:v>Sub-task</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
+<worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="true" max="1" min="1" width="8.75"/>
+    <col customWidth="true" max="2" min="2" width="6.059999942779541"/>
+    <col customWidth="true" max="3" min="3" width="10.770000457763672"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="63" t="str">
+        <v>Status</v>
+      </c>
+      <c r="B1" s="63" t="str">
+        <v>Priority</v>
+      </c>
+      <c r="C1" s="63" t="str">
+        <v>Type</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Open</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Blocker</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Bug</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>In Progress</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Task</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Resolved</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Major</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Improvement</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Closed</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Minor</v>
+      </c>
+      <c r="C5" t="str">
+        <v>New Feature</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="str">
+        <v>Trivial</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Test</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="C7" t="str">
+        <v>Sub-task</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="32" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="26" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="36" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="68" t="str">
-        <x:v>CSV / XLSX Data Schema</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="63" t="str">
-        <x:v>Column</x:v>
-      </x:c>
-      <x:c r="B3" s="63" t="str">
-        <x:v>Description</x:v>
-      </x:c>
-      <x:c r="C3" s="63" t="str">
-        <x:v>Placeholder</x:v>
-      </x:c>
-      <x:c r="D3" s="63" t="str">
-        <x:v>Required</x:v>
-      </x:c>
-      <x:c r="E3" s="63" t="str">
-        <x:v>Data Type</x:v>
-      </x:c>
-      <x:c r="F3" s="63" t="str">
-        <x:v>Notes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="73" t="str">
-        <x:v>Issue Key</x:v>
-      </x:c>
-      <x:c r="B4" s="73" t="str">
-        <x:v>Unique issue identifier</x:v>
-      </x:c>
-      <x:c r="C4" s="73" t="str">
-        <x:v>{{IssueKey}}</x:v>
-      </x:c>
-      <x:c r="D4" s="73" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="E4" s="73" t="str">
-        <x:v>Text</x:v>
-      </x:c>
-      <x:c r="F4" s="73" t="str">
-        <x:v>Primary lookup field</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="73" t="str">
-        <x:v>Summary</x:v>
-      </x:c>
-      <x:c r="B5" s="73" t="str">
-        <x:v>Short issue title</x:v>
-      </x:c>
-      <x:c r="C5" s="73" t="str">
-        <x:v>{{Summary}}</x:v>
-      </x:c>
-      <x:c r="D5" s="73" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="E5" s="73" t="str">
-        <x:v>Text</x:v>
-      </x:c>
-      <x:c r="F5" s="73" t="str"/>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="73" t="str">
-        <x:v>Type</x:v>
-      </x:c>
-      <x:c r="B6" s="73" t="str">
-        <x:v>Issue type</x:v>
-      </x:c>
-      <x:c r="C6" s="73" t="str">
-        <x:v>{{Type}}</x:v>
-      </x:c>
-      <x:c r="D6" s="73" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="E6" s="73" t="str">
-        <x:v>Enum</x:v>
-      </x:c>
-      <x:c r="F6" s="73" t="str">
-        <x:v>Bug, Task, Improvement, ...</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="73" t="str">
-        <x:v>Status</x:v>
-      </x:c>
-      <x:c r="B7" s="73" t="str">
-        <x:v>Current status</x:v>
-      </x:c>
-      <x:c r="C7" s="73" t="str">
-        <x:v>{{Status}}</x:v>
-      </x:c>
-      <x:c r="D7" s="73" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="E7" s="73" t="str">
-        <x:v>Enum</x:v>
-      </x:c>
-      <x:c r="F7" s="73" t="str">
-        <x:v>Resolved, Open, ...</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="73" t="str">
-        <x:v>Priority</x:v>
-      </x:c>
-      <x:c r="B8" s="73" t="str">
-        <x:v>Priority level</x:v>
-      </x:c>
-      <x:c r="C8" s="73" t="str">
-        <x:v>{{Priority}}</x:v>
-      </x:c>
-      <x:c r="D8" s="73" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="E8" s="73" t="str">
-        <x:v>Enum</x:v>
-      </x:c>
-      <x:c r="F8" s="73" t="str"/>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="73" t="str">
-        <x:v>Resolution</x:v>
-      </x:c>
-      <x:c r="B9" s="73" t="str">
-        <x:v>Resolution value</x:v>
-      </x:c>
-      <x:c r="C9" s="73" t="str">
-        <x:v>{{Resolution}}</x:v>
-      </x:c>
-      <x:c r="D9" s="73" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="E9" s="73" t="str">
-        <x:v>Text</x:v>
-      </x:c>
-      <x:c r="F9" s="73" t="str"/>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="73" t="str">
-        <x:v>Assignee</x:v>
-      </x:c>
-      <x:c r="B10" s="73" t="str">
-        <x:v>Assigned person</x:v>
-      </x:c>
-      <x:c r="C10" s="73" t="str">
-        <x:v>{{Assignee}}</x:v>
-      </x:c>
-      <x:c r="D10" s="73" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="E10" s="73" t="str">
-        <x:v>Text</x:v>
-      </x:c>
-      <x:c r="F10" s="73" t="str"/>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="73" t="str">
-        <x:v>Reporter</x:v>
-      </x:c>
-      <x:c r="B11" s="73" t="str">
-        <x:v>Reported by</x:v>
-      </x:c>
-      <x:c r="C11" s="73" t="str">
-        <x:v>{{Reporter}}</x:v>
-      </x:c>
-      <x:c r="D11" s="73" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="E11" s="73" t="str">
-        <x:v>Text</x:v>
-      </x:c>
-      <x:c r="F11" s="73" t="str"/>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="73" t="str">
-        <x:v>Created</x:v>
-      </x:c>
-      <x:c r="B12" s="73" t="str">
-        <x:v>Creation date/time</x:v>
-      </x:c>
-      <x:c r="C12" s="73" t="str">
-        <x:v>{{Created}}</x:v>
-      </x:c>
-      <x:c r="D12" s="73" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="E12" s="73" t="str">
-        <x:v>Datetime</x:v>
-      </x:c>
-      <x:c r="F12" s="73" t="str"/>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="73" t="str">
-        <x:v>Created Epoch</x:v>
-      </x:c>
-      <x:c r="B13" s="73" t="str">
-        <x:v>Creation epoch</x:v>
-      </x:c>
-      <x:c r="C13" s="73" t="str">
-        <x:v>{{CreatedEpoch}}</x:v>
-      </x:c>
-      <x:c r="D13" s="73" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="E13" s="73" t="str">
-        <x:v>Integer</x:v>
-      </x:c>
-      <x:c r="F13" s="73" t="str">
-        <x:v>Milliseconds UTC</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="73" t="str">
-        <x:v>Updated</x:v>
-      </x:c>
-      <x:c r="B14" s="73" t="str">
-        <x:v>Last update date/time</x:v>
-      </x:c>
-      <x:c r="C14" s="73" t="str">
-        <x:v>{{Updated}}</x:v>
-      </x:c>
-      <x:c r="D14" s="73" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="E14" s="73" t="str">
-        <x:v>Datetime</x:v>
-      </x:c>
-      <x:c r="F14" s="73" t="str"/>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="73" t="str">
-        <x:v>Updated Epoch</x:v>
-      </x:c>
-      <x:c r="B15" s="73" t="str">
-        <x:v>Last update epoch</x:v>
-      </x:c>
-      <x:c r="C15" s="73" t="str">
-        <x:v>{{UpdatedEpoch}}</x:v>
-      </x:c>
-      <x:c r="D15" s="73" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="E15" s="73" t="str">
-        <x:v>Integer</x:v>
-      </x:c>
-      <x:c r="F15" s="73" t="str">
-        <x:v>Milliseconds UTC</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="73" t="str">
-        <x:v>Resolved</x:v>
-      </x:c>
-      <x:c r="B16" s="73" t="str">
-        <x:v>Resolved date/time</x:v>
-      </x:c>
-      <x:c r="C16" s="73" t="str">
-        <x:v>{{Resolved}}</x:v>
-      </x:c>
-      <x:c r="D16" s="73" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="E16" s="73" t="str">
-        <x:v>Datetime</x:v>
-      </x:c>
-      <x:c r="F16" s="73" t="str"/>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="73" t="str">
-        <x:v>Resolved Epoch</x:v>
-      </x:c>
-      <x:c r="B17" s="73" t="str">
-        <x:v>Resolved epoch</x:v>
-      </x:c>
-      <x:c r="C17" s="73" t="str">
-        <x:v>{{ResolvedEpoch}}</x:v>
-      </x:c>
-      <x:c r="D17" s="73" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="E17" s="73" t="str">
-        <x:v>Integer</x:v>
-      </x:c>
-      <x:c r="F17" s="73" t="str">
-        <x:v>Milliseconds UTC</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="73" t="str">
-        <x:v>Description</x:v>
-      </x:c>
-      <x:c r="B18" s="73" t="str">
-        <x:v>Full issue description</x:v>
-      </x:c>
-      <x:c r="C18" s="73" t="str">
-        <x:v>{{Description}}</x:v>
-      </x:c>
-      <x:c r="D18" s="73" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="E18" s="73" t="str">
-        <x:v>Long text</x:v>
-      </x:c>
-      <x:c r="F18" s="73" t="str">
-        <x:v>Wrapped</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="73" t="str">
-        <x:v>Comments JSON</x:v>
-      </x:c>
-      <x:c r="B19" s="73" t="str">
-        <x:v>All comments serialized as JSON</x:v>
-      </x:c>
-      <x:c r="C19" s="73" t="str">
-        <x:v>{{CommentsJSON}}</x:v>
-      </x:c>
-      <x:c r="D19" s="73" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="E19" s="73" t="str">
-        <x:v>JSON</x:v>
-      </x:c>
-      <x:c r="F19" s="73" t="str">
-        <x:v>Recommended for CSV export</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A1:F1"/>
-  </x:mergeCells>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
+<worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="true" max="1" min="1" width="18"/>
+    <col customWidth="true" max="2" min="2" width="32"/>
+    <col customWidth="true" max="3" min="3" width="26"/>
+    <col customWidth="true" max="4" min="4" width="12"/>
+    <col customWidth="true" max="5" min="5" width="18"/>
+    <col customWidth="true" max="6" min="6" width="36"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="68" t="str">
+        <v>CSV / XLSX Data Schema</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="63" t="str">
+        <v>Column</v>
+      </c>
+      <c r="B3" s="63" t="str">
+        <v>Description</v>
+      </c>
+      <c r="C3" s="63" t="str">
+        <v>Placeholder</v>
+      </c>
+      <c r="D3" s="63" t="str">
+        <v>Required</v>
+      </c>
+      <c r="E3" s="63" t="str">
+        <v>Data Type</v>
+      </c>
+      <c r="F3" s="63" t="str">
+        <v>Notes</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="73" t="str">
+        <v>Issue Key</v>
+      </c>
+      <c r="B4" s="73" t="str">
+        <v>Unique issue identifier</v>
+      </c>
+      <c r="C4" s="73" t="str">
+        <v>{{IssueKey}}</v>
+      </c>
+      <c r="D4" s="73" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E4" s="73" t="str">
+        <v>Text</v>
+      </c>
+      <c r="F4" s="73" t="str">
+        <v>Primary lookup field</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="73" t="str">
+        <v>Summary</v>
+      </c>
+      <c r="B5" s="73" t="str">
+        <v>Short issue title</v>
+      </c>
+      <c r="C5" s="73" t="str">
+        <v>{{Summary}}</v>
+      </c>
+      <c r="D5" s="73" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E5" s="73" t="str">
+        <v>Text</v>
+      </c>
+      <c r="F5" s="73" t="str"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="73" t="str">
+        <v>Type</v>
+      </c>
+      <c r="B6" s="73" t="str">
+        <v>Issue type</v>
+      </c>
+      <c r="C6" s="73" t="str">
+        <v>{{Type}}</v>
+      </c>
+      <c r="D6" s="73" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E6" s="73" t="str">
+        <v>Enum</v>
+      </c>
+      <c r="F6" s="73" t="str">
+        <v>Bug, Task, Improvement, ...</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="73" t="str">
+        <v>Status</v>
+      </c>
+      <c r="B7" s="73" t="str">
+        <v>Current status</v>
+      </c>
+      <c r="C7" s="73" t="str">
+        <v>{{Status}}</v>
+      </c>
+      <c r="D7" s="73" t="str">
+        <v>No</v>
+      </c>
+      <c r="E7" s="73" t="str">
+        <v>Enum</v>
+      </c>
+      <c r="F7" s="73" t="str">
+        <v>Resolved, Open, ...</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="73" t="str">
+        <v>Priority</v>
+      </c>
+      <c r="B8" s="73" t="str">
+        <v>Priority level</v>
+      </c>
+      <c r="C8" s="73" t="str">
+        <v>{{Priority}}</v>
+      </c>
+      <c r="D8" s="73" t="str">
+        <v>No</v>
+      </c>
+      <c r="E8" s="73" t="str">
+        <v>Enum</v>
+      </c>
+      <c r="F8" s="73" t="str"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="73" t="str">
+        <v>Resolution</v>
+      </c>
+      <c r="B9" s="73" t="str">
+        <v>Resolution value</v>
+      </c>
+      <c r="C9" s="73" t="str">
+        <v>{{Resolution}}</v>
+      </c>
+      <c r="D9" s="73" t="str">
+        <v>No</v>
+      </c>
+      <c r="E9" s="73" t="str">
+        <v>Text</v>
+      </c>
+      <c r="F9" s="73" t="str"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="73" t="str">
+        <v>Assignee</v>
+      </c>
+      <c r="B10" s="73" t="str">
+        <v>Assigned person</v>
+      </c>
+      <c r="C10" s="73" t="str">
+        <v>{{Assignee}}</v>
+      </c>
+      <c r="D10" s="73" t="str">
+        <v>No</v>
+      </c>
+      <c r="E10" s="73" t="str">
+        <v>Text</v>
+      </c>
+      <c r="F10" s="73" t="str"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="73" t="str">
+        <v>Reporter</v>
+      </c>
+      <c r="B11" s="73" t="str">
+        <v>Reported by</v>
+      </c>
+      <c r="C11" s="73" t="str">
+        <v>{{Reporter}}</v>
+      </c>
+      <c r="D11" s="73" t="str">
+        <v>No</v>
+      </c>
+      <c r="E11" s="73" t="str">
+        <v>Text</v>
+      </c>
+      <c r="F11" s="73" t="str"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="73" t="str">
+        <v>Created</v>
+      </c>
+      <c r="B12" s="73" t="str">
+        <v>Creation date/time</v>
+      </c>
+      <c r="C12" s="73" t="str">
+        <v>{{Created}}</v>
+      </c>
+      <c r="D12" s="73" t="str">
+        <v>No</v>
+      </c>
+      <c r="E12" s="73" t="str">
+        <v>Datetime</v>
+      </c>
+      <c r="F12" s="73" t="str"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="73" t="str">
+        <v>Created Epoch</v>
+      </c>
+      <c r="B13" s="73" t="str">
+        <v>Creation epoch</v>
+      </c>
+      <c r="C13" s="73" t="str">
+        <v>{{CreatedEpoch}}</v>
+      </c>
+      <c r="D13" s="73" t="str">
+        <v>No</v>
+      </c>
+      <c r="E13" s="73" t="str">
+        <v>Integer</v>
+      </c>
+      <c r="F13" s="73" t="str">
+        <v>Milliseconds UTC</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="73" t="str">
+        <v>Updated</v>
+      </c>
+      <c r="B14" s="73" t="str">
+        <v>Last update date/time</v>
+      </c>
+      <c r="C14" s="73" t="str">
+        <v>{{Updated}}</v>
+      </c>
+      <c r="D14" s="73" t="str">
+        <v>No</v>
+      </c>
+      <c r="E14" s="73" t="str">
+        <v>Datetime</v>
+      </c>
+      <c r="F14" s="73" t="str"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="73" t="str">
+        <v>Updated Epoch</v>
+      </c>
+      <c r="B15" s="73" t="str">
+        <v>Last update epoch</v>
+      </c>
+      <c r="C15" s="73" t="str">
+        <v>{{UpdatedEpoch}}</v>
+      </c>
+      <c r="D15" s="73" t="str">
+        <v>No</v>
+      </c>
+      <c r="E15" s="73" t="str">
+        <v>Integer</v>
+      </c>
+      <c r="F15" s="73" t="str">
+        <v>Milliseconds UTC</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="73" t="str">
+        <v>Resolved</v>
+      </c>
+      <c r="B16" s="73" t="str">
+        <v>Resolved date/time</v>
+      </c>
+      <c r="C16" s="73" t="str">
+        <v>{{Resolved}}</v>
+      </c>
+      <c r="D16" s="73" t="str">
+        <v>No</v>
+      </c>
+      <c r="E16" s="73" t="str">
+        <v>Datetime</v>
+      </c>
+      <c r="F16" s="73" t="str"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="73" t="str">
+        <v>Resolved Epoch</v>
+      </c>
+      <c r="B17" s="73" t="str">
+        <v>Resolved epoch</v>
+      </c>
+      <c r="C17" s="73" t="str">
+        <v>{{ResolvedEpoch}}</v>
+      </c>
+      <c r="D17" s="73" t="str">
+        <v>No</v>
+      </c>
+      <c r="E17" s="73" t="str">
+        <v>Integer</v>
+      </c>
+      <c r="F17" s="73" t="str">
+        <v>Milliseconds UTC</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="73" t="str">
+        <v>Description</v>
+      </c>
+      <c r="B18" s="73" t="str">
+        <v>Full issue description</v>
+      </c>
+      <c r="C18" s="73" t="str">
+        <v>{{Description}}</v>
+      </c>
+      <c r="D18" s="73" t="str">
+        <v>No</v>
+      </c>
+      <c r="E18" s="73" t="str">
+        <v>Long text</v>
+      </c>
+      <c r="F18" s="73" t="str">
+        <v>Wrapped</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="73" t="str">
+        <v>Comments JSON</v>
+      </c>
+      <c r="B19" s="73" t="str">
+        <v>All comments serialized as JSON</v>
+      </c>
+      <c r="C19" s="73" t="str">
+        <v>{{CommentsJSON}}</v>
+      </c>
+      <c r="D19" s="73" t="str">
+        <v>No</v>
+      </c>
+      <c r="E19" s="73" t="str">
+        <v>JSON</v>
+      </c>
+      <c r="F19" s="73" t="str">
+        <v>Recommended for CSV export</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>